<commit_message>
Enhance WBGT CrewSafe SG proposal with lightning risk integration and update related documentation
</commit_message>
<xml_diff>
--- a/proposal-deliverables/WBGT-CrewSafe-SG-Product-Backlog.xlsx
+++ b/proposal-deliverables/WBGT-CrewSafe-SG-Product-Backlog.xlsx
@@ -178,10 +178,10 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -769,7 +769,7 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>US-05</t>
+          <t>US-04L</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Supervisor sees current conditions and active shift context</t>
+          <t>Lightning stop-work warning shown above WBGT</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
@@ -787,12 +787,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
+          <t>Backend (Spring Boot scheduler); NEA lightning observation API; React · React Native</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Web view uses shared backend and shows freshness</t>
+          <t>Risk state clear/advisory/stop-work; warning atop WBGT; overrides heat plan</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>US-06</t>
+          <t>US-05</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -814,32 +814,32 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>System forecasts 30 / 60-minute WBGT</t>
+          <t>Supervisor sees current conditions and active shift context</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Python ML service (FastAPI, pandas, scikit-learn / XGBoost, time-series regression)</t>
+          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Baselines measured; versioned prediction returned</t>
+          <t>Web view uses shared backend and shows freshness</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>US-07</t>
+          <t>US-06</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Evaluate the correct deterministic policy actions</t>
+          <t>System forecasts 30 / 60-minute WBGT</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
@@ -857,12 +857,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Backend (Java 21 deterministic rules engine); PostgreSQL policy config</t>
+          <t>Python ML service (FastAPI, pandas, scikit-learn / XGBoost, time-series regression)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Boundary and mixed-worker tests pass</t>
+          <t>Baselines measured; versioned prediction returned</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -874,7 +874,7 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>US-08</t>
+          <t>US-07</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Supervisor receives an explainable agent draft plan</t>
+          <t>Evaluate the correct deterministic policy actions</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
@@ -892,12 +892,12 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Agentic AI (tool-calling LLM via Spring Boot adapter, JSON-schema guarded tools)</t>
+          <t>Backend (Java 21 deterministic rules engine); PostgreSQL policy config</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>No unsupported actions; policy / model references shown</t>
+          <t>Boundary and mixed-worker tests pass</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>US-09</t>
+          <t>US-08</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -919,20 +919,20 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Supervisor approves, edits or rejects a plan</t>
+          <t>Supervisor receives an explainable agent draft plan</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Web (React); Backend (Spring Boot)</t>
+          <t>Agentic AI (tool-calling LLM via Spring Boot adapter, JSON-schema guarded tools)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Draft and final versions retained; authorization enforced</t>
+          <t>No unsupported actions; policy / model references shown</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -944,7 +944,7 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>US-10</t>
+          <t>US-09</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -954,20 +954,20 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Worker receives and acknowledges an approved action</t>
+          <t>Supervisor approves, edits or rejects a plan</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Mobile (React Native); Backend (idempotency keys); PostgreSQL</t>
+          <t>Web (React); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Only affected workers see it; idempotency works</t>
+          <t>Draft and final versions retained; authorization enforced</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -979,7 +979,7 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>US-11</t>
+          <t>US-10</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -989,20 +989,20 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Worker logs rest / hydration or raises a concern</t>
+          <t>Worker receives and acknowledges an approved action</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Mobile (React Native); Backend (Spring Boot)</t>
+          <t>Mobile (React Native); Backend (idempotency keys); PostgreSQL</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Status updates in supervisor view</t>
+          <t>Only affected workers see it; idempotency works</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>US-12</t>
+          <t>US-11</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Supervisor monitors pending, late and completed actions</t>
+          <t>Worker logs rest / hydration or raises a concern</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
+          <t>Mobile (React Native); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Live state and alert count match backend records</t>
+          <t>Status updates in supervisor view</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -1049,7 +1049,7 @@
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>US-13</t>
+          <t>US-12</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1059,32 +1059,32 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Manager views compliance and response-time charts</t>
+          <t>Supervisor monitors pending, late and completed actions</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js); Backend aggregation queries</t>
+          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Metrics verified against seeded expected values</t>
+          <t>Live state and alert count match backend records</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>US-14</t>
+          <t>US-13</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1094,20 +1094,20 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Manager views forecast accuracy and fallback status</t>
+          <t>Manager views compliance and response-time charts</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Web (Chart.js); Python ML evaluation metrics; Backend</t>
+          <t>Web (React, Chart.js); Backend aggregation queries</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Metrics match evaluation artifact</t>
+          <t>Metrics verified against seeded expected values</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1119,7 +1119,7 @@
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>US-15</t>
+          <t>US-14</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Manager exports the audit timeline</t>
+          <t>Manager views forecast accuracy and fallback status</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -1137,12 +1137,12 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Backend (CSV / PDF export); Web; PostgreSQL append-only audit</t>
+          <t>Web (Chart.js); Python ML evaluation metrics; Backend</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Export contains trace IDs, actors, rules and decisions</t>
+          <t>Metrics match evaluation artifact</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1154,7 +1154,7 @@
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>US-16</t>
+          <t>US-15</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -1164,20 +1164,20 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Safe degraded behaviour during dependency failure</t>
+          <t>Manager exports the audit timeline</t>
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Backend fallback adapters (NEA / ML / LLM); persistence forecast</t>
+          <t>Backend (CSV / PDF export); Web; PostgreSQL append-only audit</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>NEA, ML and LLM failure scenarios pass</t>
+          <t>Export contains trace IDs, actors, rules and decisions</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1189,30 +1189,30 @@
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>US-17</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>In-app reminder for an unacknowledged approved action</t>
+          <t>Safe degraded behaviour during dependency failure</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Backend (scheduler); Mobile (in-app notification)</t>
+          <t>Backend fallback adapters (NEA / ML / LLM); persistence forecast</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Reminder cannot alter instruction</t>
+          <t>NEA, ML and LLM failure scenarios pass</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1224,33 +1224,68 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>In-app reminder for an unacknowledged approved action</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Backend (scheduler); Mobile (in-app notification)</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Reminder cannot alter instruction</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>US-18</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Could</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Worker views an approved instruction in another language</t>
         </is>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Agentic AI (human-approved LLM template); Mobile (React Native)</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Human-approved template only</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Stretch</t>
         </is>
@@ -1270,7 +1305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1347,178 +1382,190 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>View current &amp; forecast risk (live conditions)</t>
+          <t>Lightning warning above WBGT (stop-work)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
+          <t>Backend (Spring Boot), NEA lightning observation API, React + React Native</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Forecast 30 / 60-minute WBGT</t>
+          <t>View current &amp; forecast risk (live conditions)</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Python ML (FastAPI, pandas, scikit-learn / XGBoost, time-series)</t>
+          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Evaluate deterministic heat policy</t>
+          <t>Forecast 30 / 60-minute WBGT</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Backend (Java 21 rules engine, PostgreSQL policy config)</t>
+          <t>Python ML (FastAPI, pandas, scikit-learn / XGBoost, time-series)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Generate explainable agent draft plan</t>
+          <t>Evaluate deterministic heat policy</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Agentic AI (tool-calling LLM via backend adapter, JSON-schema tools)</t>
+          <t>Backend (Java 21 rules engine, PostgreSQL policy config)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Approve / edit / reject plan</t>
+          <t>Generate explainable agent draft plan</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Web (React), Backend (Spring Boot)</t>
+          <t>Agentic AI (tool-calling LLM via backend adapter, JSON-schema tools)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Dispatch &amp; acknowledge worker action</t>
+          <t>Approve / edit / reject plan</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Mobile (React Native), Backend (idempotency, PostgreSQL)</t>
+          <t>Web (React), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Log rest / hydration &amp; raise safety concern</t>
+          <t>Dispatch &amp; acknowledge worker action</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mobile (React Native), Backend (Spring Boot)</t>
+          <t>Mobile (React Native), Backend (idempotency, PostgreSQL)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Monitor completion (live status board)</t>
+          <t>Log rest / hydration &amp; raise safety concern</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
+          <t>Mobile (React Native), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Compliance &amp; response-time dashboard</t>
+          <t>Monitor completion (live status board)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js), Backend aggregation</t>
+          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Model-performance dashboard</t>
+          <t>Compliance &amp; response-time dashboard</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Web (Chart.js), Python ML metrics, Backend</t>
+          <t>Web (React, Chart.js), Backend aggregation</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Export audit timeline (CSV / PDF)</t>
+          <t>Model-performance dashboard</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Backend (export service), Web, PostgreSQL append-only audit</t>
+          <t>Web (Chart.js), Python ML metrics, Backend</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Graceful degraded mode</t>
+          <t>Export audit timeline (CSV / PDF)</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Backend fallback adapters (NEA / ML / LLM)</t>
+          <t>Backend (export service), Web, PostgreSQL append-only audit</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>[Stretch] Multilingual instruction template</t>
+          <t>Graceful degraded mode</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Agentic AI (human-approved LLM template), Mobile</t>
+          <t>Backend fallback adapters (NEA / ML / LLM)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>[Cross-cutting] Cloud deployment</t>
+          <t>[Stretch] Multilingual instruction template</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Azure Container Apps, Azure Static Web Apps, Azure PostgreSQL, Blob Storage</t>
+          <t>Agentic AI (human-approved LLM template), Mobile</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
+          <t>[Cross-cutting] Cloud deployment</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>AWS: Amplify Hosting (S3 + CloudFront), ECS on Fargate, RDS for PostgreSQL, S3, Secrets Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
           <t>[Cross-cutting] DevSecOps pipeline</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>GitHub Actions CI/CD, SAST + secret scan, dependency &amp; container scanning</t>
         </is>
@@ -1538,7 +1585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1579,55 +1626,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Ingest WBGT &amp; weather (system-triggered)</t>
+          <t>Ingest WBGT, weather &amp; lightning (system-triggered)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>System (ML)</t>
+          <t>System (Lightning)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Forecast 30 / 60-minute WBGT</t>
+          <t>Classify lightning risk; raise stop-work warning above WBGT</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>System (Policy)</t>
+          <t>System (ML)</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Evaluate deterministic heat policy</t>
+          <t>Forecast 30 / 60-minute WBGT</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>System (Agent)</t>
+          <t>System (Policy)</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Draft explainable intervention plan</t>
+          <t>Evaluate deterministic heat policy</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Site Supervisor</t>
+          <t>System (Agent)</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Review &amp; approve / edit / reject plan</t>
+          <t>Draft explainable intervention plan</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1686,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Configure shift &amp; tasks</t>
+          <t>Review &amp; approve / edit / reject plan</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1698,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Monitor current &amp; forecast risk</t>
+          <t>Configure shift &amp; tasks</t>
         </is>
       </c>
     </row>
@@ -1663,19 +1710,19 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Monitor completion &amp; send approved reminder</t>
+          <t>Monitor current &amp; forecast risk</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Outdoor Worker</t>
+          <t>Site Supervisor</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Complete readiness check</t>
+          <t>Monitor completion &amp; send approved reminder</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1734,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Receive &amp; acknowledge action</t>
+          <t>Receive lightning stop-work alert &amp; seek shelter</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1746,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Log rest / hydration</t>
+          <t>Complete readiness check</t>
         </is>
       </c>
     </row>
@@ -1711,36 +1758,60 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Raise safety concern</t>
+          <t>Receive &amp; acknowledge action</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Oversight &amp; governance</t>
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Outdoor Worker</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Log rest / hydration</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
+          <t>Outdoor Worker</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Raise safety concern</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Oversight &amp; governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
           <t>Safety Manager</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Configure policy &amp; users</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Safety Manager</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>View dashboards &amp; audit / export timeline</t>
         </is>
@@ -1748,8 +1819,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A18:B18"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1921,7 +1992,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Azure Static Web Apps, Azure Container Apps, Azure PostgreSQL, Blob Storage</t>
+          <t>AWS Amplify Hosting (S3 + CloudFront), Amazon ECS on Fargate, Amazon RDS for PostgreSQL, Amazon S3, AWS Secrets Manager</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1938,7 +2009,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Structured JSON logs, correlation IDs, Application Insights</t>
+          <t>Structured JSON logs, correlation IDs, Amazon CloudWatch + AWS X-Ray</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1978,7 +2049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2157,12 +2228,12 @@
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>View current &amp; forecast risk</t>
+          <t>Lightning warning above WBGT</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Web (Chart.js), Backend</t>
+          <t>Backend, NEA lightning API, Web + Mobile</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -2175,24 +2246,28 @@
           <t>C</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr"/>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Forecast 30 / 60-minute WBGT</t>
+          <t>View current &amp; forecast risk</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Python ML (FastAPI, XGBoost)</t>
+          <t>Web (Chart.js), Backend</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -2207,12 +2282,12 @@
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Evaluate deterministic heat policy</t>
+          <t>Forecast 30 / 60-minute WBGT</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Backend rules engine</t>
+          <t>Python ML (FastAPI, XGBoost)</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -2232,12 +2307,12 @@
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Generate explainable agent draft plan</t>
+          <t>Evaluate deterministic heat policy</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Agentic AI (LLM adapter)</t>
+          <t>Backend rules engine</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -2245,7 +2320,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr"/>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="E10" s="10" t="inlineStr"/>
       <c r="F10" s="10" t="inlineStr"/>
       <c r="G10" s="10" t="inlineStr"/>
@@ -2253,12 +2332,12 @@
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Approve / edit / reject plan</t>
+          <t>Generate explainable agent draft plan</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Web, Backend</t>
+          <t>Agentic AI (LLM adapter)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -2274,12 +2353,12 @@
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Dispatch &amp; acknowledge worker action</t>
+          <t>Approve / edit / reject plan</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Mobile, Backend</t>
+          <t>Web, Backend</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -2295,7 +2374,7 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Log rest / hydration &amp; raise concern</t>
+          <t>Dispatch &amp; acknowledge worker action</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -2316,12 +2395,12 @@
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Monitor completion (live status)</t>
+          <t>Log rest / hydration &amp; raise concern</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Web, Backend</t>
+          <t>Mobile, Backend</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -2337,17 +2416,17 @@
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Compliance &amp; response-time dashboard</t>
+          <t>Monitor completion (live status)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Web (Chart.js), Backend</t>
+          <t>Web, Backend</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr"/>
@@ -2358,12 +2437,12 @@
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Model-performance dashboard</t>
+          <t>Compliance &amp; response-time dashboard</t>
         </is>
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Web, Python ML metrics</t>
+          <t>Web (Chart.js), Backend</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -2379,12 +2458,12 @@
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Export audit timeline</t>
+          <t>Model-performance dashboard</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Backend (CSV/PDF), Web</t>
+          <t>Web, Python ML metrics</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -2400,12 +2479,12 @@
     <row r="18" ht="26" customHeight="1">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Graceful degraded mode</t>
+          <t>Export audit timeline</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Backend fallback adapters</t>
+          <t>Backend (CSV/PDF), Web</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -2417,6 +2496,27 @@
       <c r="E18" s="10" t="inlineStr"/>
       <c r="F18" s="10" t="inlineStr"/>
       <c r="G18" s="10" t="inlineStr"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Graceful degraded mode</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Backend fallback adapters</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Fact-check plan, add arXiv evidence base, expand & re-sprint backlog
- Verify MOM/NEA regulatory and data claims against primary sources
- Add academic evidence base to agent (§8.4) and ML (§9.4) sections
  with SHAP explainability and forecast-reliability commitments
- Add §24.1 academic references (arXiv:2404.03310, 2603.20953,
  2607.07405, 2601.08012)
- Expand product backlog with 17 new stories (infra, DevSecOps,
  policy config, security, model card, accessibility, stretch items)
- Align sprints to AD Project schedule (Sprint 0=Wk1 .. Sprint 3=Wk4)
  and rebalance loads across sprints in plan §15 and the backlog xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proposal-deliverables/WBGT-CrewSafe-SG-Product-Backlog.xlsx
+++ b/proposal-deliverables/WBGT-CrewSafe-SG-Product-Backlog.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,6 +86,11 @@
       <color rgb="00E8873A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -120,7 +125,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -142,11 +147,44 @@
         <color rgb="00C9D4DF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9D4DF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D4DF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D4DF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D4DF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D4DF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D4DF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -205,6 +243,10 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -570,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -629,7 +671,7 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>US-01</t>
+          <t>US-19</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -639,7 +681,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Authenticate and see only my assigned site</t>
+          <t>Prepare prioritised backlog, high-level use-case diagram and UI prototype screens</t>
         </is>
       </c>
       <c r="D3" s="6" t="n">
@@ -647,59 +689,55 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Web (React, TypeScript); Mobile (React Native, Expo); Backend (Spring Boot, Spring Security, JWT); PostgreSQL</t>
+          <t>Figma / AI design tools; documentation</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>RBAC and negative authorization tests pass</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Backlog, use-case diagram and navigable mockups accepted by advisor</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>US-02</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>US-20</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Create a shift with workers, tasks and intensity</t>
-        </is>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>Web (React, MUI); Backend (Spring Boot, Spring Data JPA); PostgreSQL</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Shift validation and assignments persist</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Spike: confirm NEA WBGT/lightning feasibility and cache demo fixtures</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>NEA data.gov.sg APIs; fixture cache</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Live pull demonstrated; dated fixtures cached for offline demo</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>US-03</t>
+          <t>US-01</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -709,7 +747,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Worker views shift and submits readiness flags</t>
+          <t>Authenticate and see only my assigned site</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
@@ -717,59 +755,55 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Mobile (React Native, Expo); Backend (Spring Boot); PostgreSQL</t>
+          <t>Web (React, TypeScript); Mobile (React Native, Expo); Backend (Spring Boot, Spring Security, JWT); PostgreSQL</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Only assigned worker can submit; no medical free text</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>RBAC and negative authorization tests pass</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>US-04</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>US-02</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Ingest and store WBGT / weather with freshness</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="n">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Create a shift with workers, tasks and intensity</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>Backend (Spring Boot scheduler); NEA data.gov.sg APIs; PostgreSQL</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Live and fixture modes work; duplicate ingestion safe</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Web (React, MUI); Backend (Spring Boot, Spring Data JPA); PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Shift validation and assignments persist</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>US-04L</t>
+          <t>US-03</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -779,7 +813,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Lightning stop-work warning shown above WBGT</t>
+          <t>Worker views shift and submits readiness flags</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
@@ -787,59 +821,55 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Backend (Spring Boot scheduler); NEA lightning observation API; React · React Native</t>
+          <t>Mobile (React Native, Expo); Backend (Spring Boot); PostgreSQL</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Risk state clear/advisory/stop-work; warning atop WBGT; overrides heat plan</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Only assigned worker can submit; no medical free text</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>US-05</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>US-04</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Supervisor sees current conditions and active shift context</t>
-        </is>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Web view uses shared backend and shows freshness</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Ingest and store WBGT / weather with freshness</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Backend (Spring Boot scheduler); NEA data.gov.sg APIs; PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Live and fixture modes work; duplicate ingestion safe</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>US-06</t>
+          <t>US-04L</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -849,67 +879,63 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>System forecasts 30 / 60-minute WBGT</t>
+          <t>Lightning stop-work warning shown above WBGT</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Python ML service (FastAPI, pandas, scikit-learn / XGBoost, time-series regression)</t>
+          <t>Backend (Spring Boot scheduler); NEA lightning observation API; React · React Native</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Baselines measured; versioned prediction returned</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>Risk state clear/advisory/stop-work; warning atop WBGT; overrides heat plan</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>US-07</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Evaluate the correct deterministic policy actions</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Backend (Java 21 deterministic rules engine); PostgreSQL policy config</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Boundary and mixed-worker tests pass</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor sees current conditions and active shift context</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Web view uses shared backend and shows freshness</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>US-08</t>
+          <t>US-21</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -919,137 +945,129 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Supervisor receives an explainable agent draft plan</t>
+          <t>Provision cloud staging infrastructure and secrets management</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Agentic AI (tool-calling LLM via Spring Boot adapter, JSON-schema guarded tools)</t>
+          <t>AWS Amplify Hosting (S3 + CloudFront); ECS on Fargate; RDS for PostgreSQL; Secrets Manager</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>No unsupported actions; policy / model references shown</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>Web + mobile reach one deployed backend; no secrets in source</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>US-09</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Supervisor approves, edits or rejects a plan</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="n">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Establish CI pipeline skeleton (build, unit tests, SAST, secret scan)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Web (React); Backend (Spring Boot)</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Draft and final versions retained; authorization enforced</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Actions; SAST; secret scanning</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>PR triggers build, tests and scans; main branch protected</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>US-10</t>
+          <t>US-23</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Baseline observability: health checks, correlation IDs, structured logs</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Backend (Spring Boot Actuator); Amazon CloudWatch + X-Ray</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Health endpoints live; correlation IDs traced end-to-end</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>US-06</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Worker receives and acknowledges an approved action</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>System forecasts 30 / 60-minute WBGT</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Mobile (React Native); Backend (idempotency keys); PostgreSQL</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Only affected workers see it; idempotency works</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>US-11</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Must</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Worker logs rest / hydration or raises a concern</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>Mobile (React Native); Backend (Spring Boot)</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>Status updates in supervisor view</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Python ML service (FastAPI, pandas, scikit-learn / XGBoost, time-series regression)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Baselines measured; versioned prediction returned</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>US-12</t>
+          <t>US-07</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1059,67 +1077,63 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Supervisor monitors pending, late and completed actions</t>
+          <t>Evaluate the correct deterministic policy actions</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
+          <t>Backend (Java 21 deterministic rules engine); PostgreSQL policy config</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Live state and alert count match backend records</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>Boundary and mixed-worker tests pass</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>US-13</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>US-08</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Manager views compliance and response-time charts</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="n">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor receives an explainable agent draft plan</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>Web (React, Chart.js); Backend aggregation queries</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Metrics verified against seeded expected values</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Agentic AI (tool-calling LLM via Spring Boot adapter, JSON-schema guarded tools)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>No unsupported actions; policy / model references shown</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>US-14</t>
+          <t>US-09</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1129,7 +1143,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Manager views forecast accuracy and fallback status</t>
+          <t>Supervisor approves, edits or rejects a plan</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -1137,59 +1151,55 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Web (Chart.js); Python ML evaluation metrics; Backend</t>
+          <t>Web (React); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Metrics match evaluation artifact</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>Draft and final versions retained; authorization enforced</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>US-15</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Manager exports the audit timeline</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>Backend (CSV / PDF export); Web; PostgreSQL append-only audit</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Export contains trace IDs, actors, rules and decisions</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Worker receives and acknowledges an approved action</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (React Native); Backend (idempotency keys); PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Only affected workers see it; idempotency works</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>US-16</t>
+          <t>US-11</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1199,77 +1209,73 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Safe degraded behaviour during dependency failure</t>
+          <t>Worker logs rest / hydration or raises a concern</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Backend fallback adapters (NEA / ML / LLM); persistence forecast</t>
+          <t>Mobile (React Native); Backend (Spring Boot)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>NEA, ML and LLM failure scenarios pass</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>Status updates in supervisor view</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>US-17</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Should</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>In-app reminder for an unacknowledged approved action</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>Backend (scheduler); Mobile (in-app notification)</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>Reminder cannot alter instruction</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>US-12</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor monitors pending, late and completed actions</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Web (React, Chart.js); Backend (Spring Boot)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Live state and alert count match backend records</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>US-18</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Could</t>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Worker views an approved instruction in another language</t>
+          <t>Safety manager configures and versions the active heat policy</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
@@ -1277,23 +1283,600 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
+          <t>Web (React); Backend (Spring Boot); PostgreSQL policy_version</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Versioned catalogue with source &amp; effective date; recommendations cite version</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>US-27</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Complete DevSecOps pipeline (dependency + container scan, auto staging deploy, smoke tests)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Actions; dependency scan; container scan; staging deploy</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Pipeline scans, deploys staging and runs smoke tests</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Manager views compliance and response-time charts</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Web (React, Chart.js); Backend aggregation queries</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Metrics verified against seeded expected values</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Manager views forecast accuracy and fallback status</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Web (Chart.js); Python ML evaluation metrics; Backend</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Metrics match evaluation artifact</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Manager exports the audit timeline</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Backend (CSV / PDF export); Web; PostgreSQL append-only audit</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Export contains trace IDs, actors, rules and decisions</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Safe degraded behaviour during dependency failure</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Backend fallback adapters (NEA / ML / LLM); persistence forecast</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>NEA, ML and LLM failure scenarios pass</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>In-app reminder for an unacknowledged approved action</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Backend (scheduler); Mobile (in-app notification)</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Reminder cannot alter instruction</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>US-25</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Show readiness-check freshness and missing checks</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Mobile + Web (React); Backend (Spring Boot)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Stale or missing readiness flagged to supervisor</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>US-26</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>STPA-derived agent guardrail verification (allowlist + approval gate)</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Agentic AI adapter; Backend validation; test harness</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Unsupported-action rate zero; approval-gate bypass blocked and audited</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>US-28</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Security testing suite and remediation evidence</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Authz / injection / XSS / prompt-injection / audit-tamper tests; dependency &amp; container review</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Findings, severity, remediation and re-test documented; no unresolved high/critical</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>US-29</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>ML model card with SHAP explainability and forecast-reliability</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Python ML (SHAP); model-card document</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Card includes SHAP drivers, calibration and per-band error</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>US-30</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Admin manages users, roles, sites and integrations</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Web (React); Backend (Spring Security); PostgreSQL</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Admin CRUD with RBAC; every change audited</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>US-31</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Accessibility and performance checks (WCAG 2.1 AA basics; p95 latency)</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Web + Mobile; axe / Lighthouse; load test</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>WCAG AA basics met; read p95 &lt;1s, write p95 &lt;2s</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>US-18</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Worker views an approved instruction in another language</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
           <t>Agentic AI (human-approved LLM template); Mobile (React Native)</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>Human-approved template only</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G34" s="6" t="inlineStr">
         <is>
           <t>Stretch</t>
         </is>
       </c>
     </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>US-32</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>QR check-in at a simulated rest zone</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (Expo Camera); Backend</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Scan logs rest at zone; event audited</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>US-33</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Multi-site management view</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Web (React); Backend (Spring Boot)</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Manager switches and compares multiple sites</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="42" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>US-34</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Supervisor-entered local WBGT reading with source &amp; timestamp</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Web + Mobile; Backend (Spring Boot)</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Manual reading stored with source/time; no station-equivalence claim</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>US-35</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Push notifications via Firebase Cloud Messaging</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (Expo + FCM); Backend</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Approved action pushes to worker device</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="40" customHeight="1">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Sprint schedule (per AD Project Instructions): Sprint 0 = Week 1 (Inception &amp; Requirements) · Sprint 1 = Week 2 (Design &amp; Prototyping / infrastructure) · Sprint 2 = Week 3 (Development / MVP + DevSecOps) · Sprint 3 = Week 4 (Development, quality, security, demo) · Stretch = post-MVP, only after all Must stories pass.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1305,7 +1888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1344,12 +1927,12 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Configure shift, tasks &amp; assignments</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Web (React, MUI), Backend (Spring Boot, Spring Data JPA, PostgreSQL)</t>
         </is>
@@ -1368,12 +1951,12 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Ingest WBGT &amp; weather with freshness</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Backend (Spring Boot scheduler), NEA data.gov.sg APIs, PostgreSQL</t>
         </is>
@@ -1392,12 +1975,12 @@
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>View current &amp; forecast risk (live conditions)</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Web (React, Chart.js), Backend (Spring Boot)</t>
         </is>
@@ -1416,12 +1999,12 @@
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Evaluate deterministic heat policy</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Backend (Java 21 rules engine, PostgreSQL policy config)</t>
         </is>
@@ -1430,142 +2013,286 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
+          <t>Configure &amp; version heat policy</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Web (React), Backend (Spring Boot), PostgreSQL policy_version</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
           <t>Generate explainable agent draft plan</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Agentic AI (tool-calling LLM via backend adapter, JSON-schema tools)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Approve / edit / reject plan</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Web (React), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Dispatch &amp; acknowledge worker action</t>
+          <t>Agent guardrail verification (STPA, allowlist, approval gate)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mobile (React Native), Backend (idempotency, PostgreSQL)</t>
+          <t>Agentic AI adapter, Backend validation, test harness</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Log rest / hydration &amp; raise safety concern</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Mobile (React Native), Backend (Spring Boot)</t>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Approve / edit / reject plan</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Web (React), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Monitor completion (live status board)</t>
+          <t>Dispatch &amp; acknowledge worker action</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
+          <t>Mobile (React Native), Backend (idempotency, PostgreSQL)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Compliance &amp; response-time dashboard</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Web (React, Chart.js), Backend aggregation</t>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Log rest / hydration &amp; raise safety concern</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (React Native), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Model-performance dashboard</t>
+          <t>Readiness-check freshness &amp; missing-check indicators</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Web (Chart.js), Python ML metrics, Backend</t>
+          <t>Mobile + Web (React), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Export audit timeline (CSV / PDF)</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Backend (export service), Web, PostgreSQL append-only audit</t>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Monitor completion (live status board)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Web (React, Chart.js), Backend (Spring Boot)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>Graceful degraded mode</t>
+          <t>Compliance &amp; response-time dashboard</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Backend fallback adapters (NEA / ML / LLM)</t>
+          <t>Web (React, Chart.js), Backend aggregation</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>[Stretch] Multilingual instruction template</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Agentic AI (human-approved LLM template), Mobile</t>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Model-performance dashboard</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Web (Chart.js), Python ML metrics, Backend</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
+          <t>ML model card (SHAP explainability, reliability)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Python ML (SHAP), model-card documentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Export audit timeline (CSV / PDF)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Backend (export service), Web, PostgreSQL append-only audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Graceful degraded mode</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Backend fallback adapters (NEA / ML / LLM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Observability &amp; health monitoring</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Backend (Spring Boot Actuator), CloudWatch + X-Ray</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Security testing &amp; remediation evidence</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>OWASP-style tests (authz, injection, XSS, prompt-injection, audit-tamper), dependency &amp; container scanning</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Accessibility &amp; performance</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Web + Mobile, axe / Lighthouse, load test (WCAG 2.1 AA basics; p95 latency)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Admin: users, roles, sites &amp; integrations</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Web (React), Backend (Spring Security), PostgreSQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>[Stretch] Multilingual instruction template</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Agentic AI (human-approved LLM template), Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>[Stretch] QR rest-zone check-in</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (Expo Camera), Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>[Stretch] Multi-site management view</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Web (React), Backend (Spring Boot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>[Stretch] Supervisor-entered local WBGT reading</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Web + Mobile, Backend (Spring Boot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>[Stretch] Push notifications (Firebase Cloud Messaging)</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Mobile (Expo + FCM), Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
           <t>[Cross-cutting] Cloud deployment</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>AWS: Amplify Hosting (S3 + CloudFront), ECS on Fargate, RDS for PostgreSQL, S3, Secrets Manager</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>[Cross-cutting] DevSecOps pipeline</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>GitHub Actions CI/CD, SAST + secret scan, dependency &amp; container scanning</t>
         </is>
@@ -1617,6 +2344,7 @@
           <t>Core observe → decide → approve → dispatch → acknowledge → audit loop</t>
         </is>
       </c>
+      <c r="B3" s="21" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -1792,6 +2520,7 @@
           <t>Oversight &amp; governance</t>
         </is>
       </c>
+      <c r="B18" s="21" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
@@ -2049,7 +2778,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2116,10 +2845,8 @@
           <t>Web + Mobile + Backend, PostgreSQL</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C3" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
@@ -2139,33 +2866,31 @@
       <c r="G3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Configure shift, tasks &amp; assignments</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Web, Backend, PostgreSQL</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="C4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr"/>
-      <c r="G4" s="10" t="inlineStr"/>
+      <c r="F4" s="17" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
@@ -2178,52 +2903,48 @@
           <t>Mobile, Backend, PostgreSQL</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C5" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr"/>
+      <c r="F5" s="17" t="inlineStr"/>
       <c r="G5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Ingest WBGT &amp; weather with freshness</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Backend, NEA APIs, PostgreSQL</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="C6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr"/>
-      <c r="G6" s="10" t="inlineStr"/>
+      <c r="F6" s="17" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
@@ -2236,287 +2957,456 @@
           <t>Backend, NEA lightning API, Web + Mobile</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C7" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="F7" s="17" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>View current &amp; forecast risk</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Web (Chart.js), Backend</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="C8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr"/>
-      <c r="F8" s="10" t="inlineStr"/>
-      <c r="G8" s="10" t="inlineStr"/>
+      <c r="E8" s="16" t="inlineStr"/>
+      <c r="F8" s="17" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Forecast 30 / 60-minute WBGT</t>
+          <t>Provision cloud staging &amp; secrets</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Python ML (FastAPI, XGBoost)</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>AWS Amplify / ECS / RDS / Secrets Manager</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Evaluate deterministic heat policy</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Backend rules engine</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>CI pipeline skeleton (build/test/SAST/secret)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr"/>
-      <c r="F10" s="10" t="inlineStr"/>
-      <c r="G10" s="10" t="inlineStr"/>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Generate explainable agent draft plan</t>
+          <t>Observability (health, correlation IDs, logs)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Agentic AI (LLM adapter)</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr"/>
+          <t>Backend Actuator, CloudWatch + X-Ray</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr"/>
+      <c r="F11" s="17" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Approve / edit / reject plan</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Web, Backend</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr"/>
-      <c r="F12" s="10" t="inlineStr"/>
-      <c r="G12" s="10" t="inlineStr"/>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Forecast 30 / 60-minute WBGT</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Python ML (FastAPI, XGBoost)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr"/>
+      <c r="F12" s="17" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Dispatch &amp; acknowledge worker action</t>
+          <t>Evaluate deterministic heat policy</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mobile, Backend</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
+          <t>Backend rules engine</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr"/>
+      <c r="F13" s="17" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>Log rest / hydration &amp; raise concern</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Mobile, Backend</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="inlineStr"/>
-      <c r="E14" s="10" t="inlineStr"/>
-      <c r="F14" s="10" t="inlineStr"/>
-      <c r="G14" s="10" t="inlineStr"/>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Configure &amp; version heat policy</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Web, Backend, PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr"/>
+      <c r="F14" s="17" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Monitor completion (live status)</t>
+          <t>Generate explainable agent draft plan</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
+          <t>Agentic AI (LLM adapter)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="16" t="inlineStr"/>
+      <c r="E15" s="16" t="inlineStr"/>
+      <c r="F15" s="17" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Approve / edit / reject plan</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
           <t>Web, Backend</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr"/>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="6" t="inlineStr"/>
-      <c r="G15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Compliance &amp; response-time dashboard</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Web (Chart.js), Backend</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D16" s="10" t="inlineStr"/>
-      <c r="E16" s="10" t="inlineStr"/>
-      <c r="F16" s="10" t="inlineStr"/>
-      <c r="G16" s="10" t="inlineStr"/>
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="16" t="inlineStr"/>
+      <c r="E16" s="16" t="inlineStr"/>
+      <c r="F16" s="17" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="26" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Model-performance dashboard</t>
+          <t>Dispatch &amp; acknowledge worker action</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Web, Python ML metrics</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="6" t="inlineStr"/>
+          <t>Mobile, Backend</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr"/>
+      <c r="E17" s="16" t="inlineStr"/>
+      <c r="F17" s="17" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="14" t="inlineStr">
-        <is>
-          <t>Export audit timeline</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Backend (CSV/PDF), Web</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr"/>
-      <c r="E18" s="10" t="inlineStr"/>
-      <c r="F18" s="10" t="inlineStr"/>
-      <c r="G18" s="10" t="inlineStr"/>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Log rest / hydration &amp; raise concern</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mobile, Backend</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="16" t="inlineStr"/>
+      <c r="E18" s="16" t="inlineStr"/>
+      <c r="F18" s="17" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="26" customHeight="1">
       <c r="A19" s="13" t="inlineStr">
         <is>
+          <t>Monitor completion (live status)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Web, Backend</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr"/>
+      <c r="E19" s="16" t="inlineStr"/>
+      <c r="F19" s="17" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Complete DevSecOps pipeline (dep/container scan, staging deploy)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="16" t="inlineStr"/>
+      <c r="E20" s="16" t="inlineStr"/>
+      <c r="F20" s="17" t="inlineStr"/>
+      <c r="G20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Compliance &amp; response-time dashboard</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Web (Chart.js), Backend</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="16" t="inlineStr"/>
+      <c r="E21" s="16" t="inlineStr"/>
+      <c r="F21" s="17" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Model-performance dashboard</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Web, Python ML metrics</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" s="16" t="inlineStr"/>
+      <c r="E22" s="16" t="inlineStr"/>
+      <c r="F22" s="17" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Export audit timeline</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Backend (CSV/PDF), Web</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="16" t="inlineStr"/>
+      <c r="E23" s="16" t="inlineStr"/>
+      <c r="F23" s="17" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
           <t>Graceful degraded mode</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Backend fallback adapters</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr"/>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
+      <c r="C24" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="16" t="inlineStr"/>
+      <c r="E24" s="16" t="inlineStr"/>
+      <c r="F24" s="17" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Security testing &amp; remediation</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>OWASP-style tests, dependency &amp; container scan</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="16" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr"/>
+      <c r="F25" s="17" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>ML model card (SHAP, reliability)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Python ML (SHAP), documentation</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="16" t="inlineStr"/>
+      <c r="E26" s="16" t="inlineStr"/>
+      <c r="F26" s="17" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Admin: users, roles, sites &amp; integrations</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Web, Backend (Spring Security)</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr"/>
+      <c r="E27" s="16" t="inlineStr"/>
+      <c r="F27" s="17" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="26" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>Accessibility &amp; performance checks</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>axe / Lighthouse, load test</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" s="16" t="inlineStr"/>
+      <c r="E28" s="16" t="inlineStr"/>
+      <c r="F28" s="17" t="inlineStr"/>
+      <c r="G28" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>